<commit_message>
Digikey (receiver and transmitter) and LCSC (receiver BOM) added
</commit_message>
<xml_diff>
--- a/Hardware-Designing/_Documents/Deliverables-(Transmitter)/BOM/Martin_BOM_DigiKey-(Transmitter).xlsx
+++ b/Hardware-Designing/_Documents/Deliverables-(Transmitter)/BOM/Martin_BOM_DigiKey-(Transmitter).xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\MartinS\Martin_Smith\Hardware-Designing\_Documents\Deliverables-(Transmitter)\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Martin_Smith\Hardware-Designing\_Documents\Deliverables-(Transmitter)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23699906-45D6-4C0B-A8AE-0F5F34968B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="1560" yWindow="900" windowWidth="10335" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -279,7 +280,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -900,6 +901,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="6" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -925,12 +932,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1034,6 +1035,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1069,6 +1087,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1244,7 +1279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1268,23 +1303,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="65"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="67"/>
       <c r="P1" s="42"/>
       <c r="Q1" s="39"/>
     </row>
@@ -1345,7 +1380,7 @@
       <c r="A3" s="59">
         <v>1</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="69" t="s">
         <v>38</v>
       </c>
       <c r="C3" s="52" t="s">
@@ -1376,7 +1411,7 @@
         <f>J3*5</f>
         <v>5</v>
       </c>
-      <c r="L3" s="70" t="s">
+      <c r="L3" s="61" t="s">
         <v>14</v>
       </c>
       <c r="M3" s="15">
@@ -1399,7 +1434,7 @@
       <c r="A4" s="59">
         <v>2</v>
       </c>
-      <c r="B4" s="68"/>
+      <c r="B4" s="70"/>
       <c r="C4" s="54" t="s">
         <v>50</v>
       </c>
@@ -1451,7 +1486,7 @@
       <c r="A5" s="9">
         <v>3</v>
       </c>
-      <c r="B5" s="68"/>
+      <c r="B5" s="70"/>
       <c r="C5" s="54" t="s">
         <v>56</v>
       </c>
@@ -1503,7 +1538,7 @@
       <c r="A6" s="59">
         <v>4</v>
       </c>
-      <c r="B6" s="68"/>
+      <c r="B6" s="70"/>
       <c r="C6" s="54" t="s">
         <v>22</v>
       </c>
@@ -1555,7 +1590,7 @@
       <c r="A7" s="59">
         <v>5</v>
       </c>
-      <c r="B7" s="68"/>
+      <c r="B7" s="70"/>
       <c r="C7" s="54" t="s">
         <v>61</v>
       </c>
@@ -1607,7 +1642,7 @@
       <c r="A8" s="59">
         <v>18</v>
       </c>
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="69" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="52" t="s">
@@ -1638,7 +1673,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L8" s="70" t="s">
+      <c r="L8" s="61" t="s">
         <v>14</v>
       </c>
       <c r="M8" s="25">
@@ -1661,7 +1696,7 @@
       <c r="A9" s="59">
         <v>19</v>
       </c>
-      <c r="B9" s="68"/>
+      <c r="B9" s="70"/>
       <c r="C9" s="54" t="s">
         <v>69</v>
       </c>
@@ -1713,7 +1748,7 @@
       <c r="A10" s="59">
         <v>20</v>
       </c>
-      <c r="B10" s="68"/>
+      <c r="B10" s="70"/>
       <c r="C10" s="54" t="s">
         <v>72</v>
       </c>
@@ -1765,7 +1800,7 @@
       <c r="A11" s="59">
         <v>34</v>
       </c>
-      <c r="B11" s="67" t="s">
+      <c r="B11" s="69" t="s">
         <v>40</v>
       </c>
       <c r="C11" s="53" t="s">
@@ -1774,7 +1809,7 @@
       <c r="D11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="71" t="s">
+      <c r="E11" s="62" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="30" t="s">
@@ -1796,7 +1831,7 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L11" s="70" t="s">
+      <c r="L11" s="61" t="s">
         <v>78</v>
       </c>
       <c r="M11" s="25">
@@ -1819,7 +1854,7 @@
       <c r="A12" s="59">
         <v>35</v>
       </c>
-      <c r="B12" s="68"/>
+      <c r="B12" s="70"/>
       <c r="C12" s="54" t="s">
         <v>79</v>
       </c>
@@ -1873,7 +1908,7 @@
       <c r="A13" s="59">
         <v>44</v>
       </c>
-      <c r="B13" s="69"/>
+      <c r="B13" s="71"/>
       <c r="C13" s="54" t="s">
         <v>82</v>
       </c>
@@ -1925,7 +1960,7 @@
       <c r="A14" s="59">
         <v>46</v>
       </c>
-      <c r="B14" s="69"/>
+      <c r="B14" s="71"/>
       <c r="C14" s="34" t="s">
         <v>45</v>
       </c>
@@ -1983,12 +2018,12 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15"/>
-      <c r="J15" s="66" t="s">
+      <c r="J15" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="K15" s="66"/>
-      <c r="L15" s="66"/>
-      <c r="M15" s="66"/>
+      <c r="K15" s="68"/>
+      <c r="L15" s="68"/>
+      <c r="M15" s="68"/>
       <c r="N15" s="2"/>
       <c r="O15" s="5"/>
       <c r="P15" s="3">
@@ -2007,12 +2042,12 @@
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16"/>
-      <c r="J16" s="61" t="s">
+      <c r="J16" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
+      <c r="K16" s="63"/>
+      <c r="L16" s="63"/>
+      <c r="M16" s="63"/>
       <c r="N16" s="4">
         <f>SUM(N3:N14)</f>
         <v>6.2099999999999991</v>
@@ -2103,17 +2138,17 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L4" r:id="rId1"/>
-    <hyperlink ref="L5" r:id="rId2"/>
-    <hyperlink ref="L6" r:id="rId3"/>
-    <hyperlink ref="L7" r:id="rId4"/>
-    <hyperlink ref="L13" r:id="rId5"/>
-    <hyperlink ref="L8" r:id="rId6"/>
-    <hyperlink ref="L9" r:id="rId7"/>
-    <hyperlink ref="L10" r:id="rId8"/>
-    <hyperlink ref="L11" r:id="rId9"/>
-    <hyperlink ref="L12" r:id="rId10"/>
-    <hyperlink ref="L3" r:id="rId11"/>
+    <hyperlink ref="L4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="L5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="L6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="L7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="L13" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="L8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="L9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="L10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="L11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="L12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="L3" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId12"/>

</xml_diff>

<commit_message>
LCSC transmitter BOM added
</commit_message>
<xml_diff>
--- a/Hardware-Designing/_Documents/Deliverables-(Transmitter)/BOM/Martin_BOM_DigiKey-(Transmitter).xlsx
+++ b/Hardware-Designing/_Documents/Deliverables-(Transmitter)/BOM/Martin_BOM_DigiKey-(Transmitter).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Martin_Smith\Hardware-Designing\_Documents\Deliverables-(Transmitter)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23699906-45D6-4C0B-A8AE-0F5F34968B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48002CB-ABD7-481D-945D-6F606705C09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="900" windowWidth="10335" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7470" yWindow="645" windowWidth="10335" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="86">
   <si>
     <t>S. No.</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t>TE Connectivity</t>
+  </si>
+  <si>
+    <t>Connectors</t>
   </si>
 </sst>
 </file>
@@ -431,7 +434,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -721,6 +724,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -731,7 +747,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="2" applyBorder="1"/>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -931,7 +947,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1908,7 +1927,9 @@
       <c r="A13" s="59">
         <v>44</v>
       </c>
-      <c r="B13" s="71"/>
+      <c r="B13" s="71" t="s">
+        <v>85</v>
+      </c>
       <c r="C13" s="54" t="s">
         <v>82</v>
       </c>
@@ -1960,7 +1981,7 @@
       <c r="A14" s="59">
         <v>46</v>
       </c>
-      <c r="B14" s="71"/>
+      <c r="B14" s="72"/>
       <c r="C14" s="34" t="s">
         <v>45</v>
       </c>

</xml_diff>